<commit_message>
H2_N2 Höchst Preis für Stickstoff
H2_N2 Höchst Preis für Stickstoff von Michi übernehmen -> Preis in betroffenen Ammoniak Modellen auf 0,2 gesetzt und Pipeline Modell archiviert
</commit_message>
<xml_diff>
--- a/Ammoniak/Ammoniak_Brownfield_H2_N2_HB_Höchst/Datenbank.xlsx
+++ b/Ammoniak/Ammoniak_Brownfield_H2_N2_HB_Höchst/Datenbank.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Ammoniak\Ammoniak_Brownfield_H2_N2_FT_Höchst\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Ammoniak\Ammoniak_Brownfield_H2_N2_HB_Höchst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E71F4327-B46A-4F20-9CFE-C1BB2B498537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFEE9695-3B9B-47E4-906C-62E0B154718A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1344,6 +1344,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1389,26 +1392,17 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1419,33 +1413,39 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1804,10 +1804,10 @@
       <c r="G1" s="6"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="81" t="s">
+      <c r="B2" s="84" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -1824,8 +1824,8 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="71"/>
-      <c r="B3" s="82"/>
+      <c r="A3" s="74"/>
+      <c r="B3" s="85"/>
       <c r="C3" t="s">
         <v>102</v>
       </c>
@@ -1840,8 +1840,8 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="71"/>
-      <c r="B4" s="82"/>
+      <c r="A4" s="74"/>
+      <c r="B4" s="85"/>
       <c r="C4" t="s">
         <v>12</v>
       </c>
@@ -1856,8 +1856,8 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="71"/>
-      <c r="B5" s="82"/>
+      <c r="A5" s="74"/>
+      <c r="B5" s="85"/>
       <c r="C5" t="s">
         <v>13</v>
       </c>
@@ -1872,8 +1872,8 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="71"/>
-      <c r="B6" s="82"/>
+      <c r="A6" s="74"/>
+      <c r="B6" s="85"/>
       <c r="C6" t="s">
         <v>15</v>
       </c>
@@ -1888,8 +1888,8 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="71"/>
-      <c r="B7" s="82"/>
+      <c r="A7" s="74"/>
+      <c r="B7" s="85"/>
       <c r="C7" t="s">
         <v>17</v>
       </c>
@@ -1904,8 +1904,8 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="71"/>
-      <c r="B8" s="83" t="s">
+      <c r="A8" s="74"/>
+      <c r="B8" s="86" t="s">
         <v>3</v>
       </c>
       <c r="C8" s="4" t="s">
@@ -1922,8 +1922,8 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="71"/>
-      <c r="B9" s="82"/>
+      <c r="A9" s="74"/>
+      <c r="B9" s="85"/>
       <c r="C9" t="s">
         <v>105</v>
       </c>
@@ -1938,41 +1938,41 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="71"/>
-      <c r="B10" s="82"/>
+      <c r="A10" s="74"/>
+      <c r="B10" s="85"/>
       <c r="C10" t="s">
         <v>12</v>
       </c>
       <c r="D10" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="103">
+      <c r="E10" s="70">
         <v>0</v>
       </c>
-      <c r="F10" s="103" t="s">
+      <c r="F10" s="70" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="71"/>
-      <c r="B11" s="82"/>
+      <c r="A11" s="74"/>
+      <c r="B11" s="85"/>
       <c r="C11" t="s">
         <v>13</v>
       </c>
       <c r="D11" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="104">
+      <c r="E11" s="71">
         <f>0.05*9070</f>
         <v>453.5</v>
       </c>
-      <c r="F11" s="105" t="s">
+      <c r="F11" s="72" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="71"/>
-      <c r="B12" s="82"/>
+      <c r="A12" s="74"/>
+      <c r="B12" s="85"/>
       <c r="C12" t="s">
         <v>110</v>
       </c>
@@ -1987,8 +1987,8 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="71"/>
-      <c r="B13" s="82"/>
+      <c r="A13" s="74"/>
+      <c r="B13" s="85"/>
       <c r="C13" t="s">
         <v>109</v>
       </c>
@@ -2003,8 +2003,8 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="71"/>
-      <c r="B14" s="82"/>
+      <c r="A14" s="74"/>
+      <c r="B14" s="85"/>
       <c r="C14" t="s">
         <v>15</v>
       </c>
@@ -2019,8 +2019,8 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="71"/>
-      <c r="B15" s="84"/>
+      <c r="A15" s="74"/>
+      <c r="B15" s="87"/>
       <c r="C15" s="5" t="s">
         <v>17</v>
       </c>
@@ -2035,8 +2035,8 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="71"/>
-      <c r="B16" s="75" t="s">
+      <c r="A16" s="74"/>
+      <c r="B16" s="78" t="s">
         <v>4</v>
       </c>
       <c r="C16" t="s">
@@ -2054,8 +2054,8 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="71"/>
-      <c r="B17" s="75"/>
+      <c r="A17" s="74"/>
+      <c r="B17" s="78"/>
       <c r="C17" t="s">
         <v>12</v>
       </c>
@@ -2070,8 +2070,8 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="71"/>
-      <c r="B18" s="75"/>
+      <c r="A18" s="74"/>
+      <c r="B18" s="78"/>
       <c r="C18" t="s">
         <v>13</v>
       </c>
@@ -2086,8 +2086,8 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="71"/>
-      <c r="B19" s="75"/>
+      <c r="A19" s="74"/>
+      <c r="B19" s="78"/>
       <c r="C19" t="s">
         <v>15</v>
       </c>
@@ -2102,8 +2102,8 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="71"/>
-      <c r="B20" s="75"/>
+      <c r="A20" s="74"/>
+      <c r="B20" s="78"/>
       <c r="C20" t="s">
         <v>17</v>
       </c>
@@ -2118,10 +2118,10 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="70" t="s">
+      <c r="A21" s="73" t="s">
         <v>85</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="B21" s="77" t="s">
         <v>5</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -2138,8 +2138,8 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="71"/>
-      <c r="B22" s="75"/>
+      <c r="A22" s="74"/>
+      <c r="B22" s="78"/>
       <c r="C22" t="s">
         <v>13</v>
       </c>
@@ -2154,8 +2154,8 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="71"/>
-      <c r="B23" s="75"/>
+      <c r="A23" s="74"/>
+      <c r="B23" s="78"/>
       <c r="C23" t="s">
         <v>15</v>
       </c>
@@ -2170,8 +2170,8 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="71"/>
-      <c r="B24" s="75"/>
+      <c r="A24" s="74"/>
+      <c r="B24" s="78"/>
       <c r="C24" t="s">
         <v>22</v>
       </c>
@@ -2186,8 +2186,8 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="71"/>
-      <c r="B25" s="75"/>
+      <c r="A25" s="74"/>
+      <c r="B25" s="78"/>
       <c r="C25" t="s">
         <v>47</v>
       </c>
@@ -2202,8 +2202,8 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="71"/>
-      <c r="B26" s="75"/>
+      <c r="A26" s="74"/>
+      <c r="B26" s="78"/>
       <c r="C26" t="s">
         <v>48</v>
       </c>
@@ -2218,8 +2218,8 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="71"/>
-      <c r="B27" s="75"/>
+      <c r="A27" s="74"/>
+      <c r="B27" s="78"/>
       <c r="C27" t="s">
         <v>17</v>
       </c>
@@ -2234,8 +2234,8 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="71"/>
-      <c r="B28" s="75"/>
+      <c r="A28" s="74"/>
+      <c r="B28" s="78"/>
       <c r="C28" t="s">
         <v>114</v>
       </c>
@@ -2250,8 +2250,8 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="71"/>
-      <c r="B29" s="76" t="s">
+      <c r="A29" s="74"/>
+      <c r="B29" s="79" t="s">
         <v>258</v>
       </c>
       <c r="C29" s="4" t="s">
@@ -2268,8 +2268,8 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="71"/>
-      <c r="B30" s="79"/>
+      <c r="A30" s="74"/>
+      <c r="B30" s="82"/>
       <c r="C30" s="51" t="s">
         <v>23</v>
       </c>
@@ -2285,8 +2285,8 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="71"/>
-      <c r="B31" s="79"/>
+      <c r="A31" s="74"/>
+      <c r="B31" s="82"/>
       <c r="C31" s="51" t="s">
         <v>18</v>
       </c>
@@ -2301,8 +2301,8 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="71"/>
-      <c r="B32" s="79"/>
+      <c r="A32" s="74"/>
+      <c r="B32" s="82"/>
       <c r="C32" s="51" t="s">
         <v>19</v>
       </c>
@@ -2317,8 +2317,8 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="71"/>
-      <c r="B33" s="79"/>
+      <c r="A33" s="74"/>
+      <c r="B33" s="82"/>
       <c r="C33" s="51" t="s">
         <v>47</v>
       </c>
@@ -2333,8 +2333,8 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="71"/>
-      <c r="B34" s="79"/>
+      <c r="A34" s="74"/>
+      <c r="B34" s="82"/>
       <c r="C34" s="51" t="s">
         <v>48</v>
       </c>
@@ -2349,8 +2349,8 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="71"/>
-      <c r="B35" s="79"/>
+      <c r="A35" s="74"/>
+      <c r="B35" s="82"/>
       <c r="C35" s="51" t="s">
         <v>115</v>
       </c>
@@ -2365,8 +2365,8 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="71"/>
-      <c r="B36" s="79"/>
+      <c r="A36" s="74"/>
+      <c r="B36" s="82"/>
       <c r="C36" s="51" t="s">
         <v>114</v>
       </c>
@@ -2381,8 +2381,8 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="71"/>
-      <c r="B37" s="79"/>
+      <c r="A37" s="74"/>
+      <c r="B37" s="82"/>
       <c r="C37" s="51" t="s">
         <v>15</v>
       </c>
@@ -2397,8 +2397,8 @@
       </c>
     </row>
     <row r="38" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="72"/>
-      <c r="B38" s="80"/>
+      <c r="A38" s="75"/>
+      <c r="B38" s="83"/>
       <c r="C38" s="14" t="s">
         <v>17</v>
       </c>
@@ -2413,7 +2413,7 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="70" t="s">
+      <c r="A39" s="73" t="s">
         <v>86</v>
       </c>
       <c r="B39" s="57" t="s">
@@ -2433,7 +2433,7 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="73"/>
+      <c r="A40" s="76"/>
       <c r="B40" s="67" t="s">
         <v>302</v>
       </c>
@@ -2444,14 +2444,14 @@
         <v>304</v>
       </c>
       <c r="E40" s="69">
-        <v>18</v>
+        <v>0.2</v>
       </c>
       <c r="F40" s="68" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="73"/>
+      <c r="A41" s="76"/>
       <c r="B41" s="60" t="s">
         <v>299</v>
       </c>
@@ -2469,8 +2469,8 @@
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="71"/>
-      <c r="B42" s="76" t="s">
+      <c r="A42" s="74"/>
+      <c r="B42" s="79" t="s">
         <v>6</v>
       </c>
       <c r="C42" s="4" t="s">
@@ -2487,8 +2487,8 @@
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="71"/>
-      <c r="B43" s="75"/>
+      <c r="A43" s="74"/>
+      <c r="B43" s="78"/>
       <c r="C43" t="s">
         <v>12</v>
       </c>
@@ -2503,8 +2503,8 @@
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="71"/>
-      <c r="B44" s="75"/>
+      <c r="A44" s="74"/>
+      <c r="B44" s="78"/>
       <c r="C44" t="s">
         <v>19</v>
       </c>
@@ -2519,8 +2519,8 @@
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="71"/>
-      <c r="B45" s="75"/>
+      <c r="A45" s="74"/>
+      <c r="B45" s="78"/>
       <c r="C45" t="s">
         <v>20</v>
       </c>
@@ -2535,8 +2535,8 @@
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="71"/>
-      <c r="B46" s="75"/>
+      <c r="A46" s="74"/>
+      <c r="B46" s="78"/>
       <c r="C46" t="s">
         <v>15</v>
       </c>
@@ -2551,8 +2551,8 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="71"/>
-      <c r="B47" s="75"/>
+      <c r="A47" s="74"/>
+      <c r="B47" s="78"/>
       <c r="C47" t="s">
         <v>82</v>
       </c>
@@ -2567,8 +2567,8 @@
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="71"/>
-      <c r="B48" s="77"/>
+      <c r="A48" s="74"/>
+      <c r="B48" s="80"/>
       <c r="C48" s="5" t="s">
         <v>17</v>
       </c>
@@ -2583,8 +2583,8 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="71"/>
-      <c r="B49" s="76" t="s">
+      <c r="A49" s="74"/>
+      <c r="B49" s="79" t="s">
         <v>7</v>
       </c>
       <c r="C49" s="4" t="s">
@@ -2601,8 +2601,8 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="71"/>
-      <c r="B50" s="75"/>
+      <c r="A50" s="74"/>
+      <c r="B50" s="78"/>
       <c r="C50" t="s">
         <v>12</v>
       </c>
@@ -2617,8 +2617,8 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="71"/>
-      <c r="B51" s="75"/>
+      <c r="A51" s="74"/>
+      <c r="B51" s="78"/>
       <c r="C51" t="s">
         <v>19</v>
       </c>
@@ -2633,8 +2633,8 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="71"/>
-      <c r="B52" s="75"/>
+      <c r="A52" s="74"/>
+      <c r="B52" s="78"/>
       <c r="C52" t="s">
         <v>20</v>
       </c>
@@ -2649,8 +2649,8 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="71"/>
-      <c r="B53" s="75"/>
+      <c r="A53" s="74"/>
+      <c r="B53" s="78"/>
       <c r="C53" t="s">
         <v>15</v>
       </c>
@@ -2665,8 +2665,8 @@
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="71"/>
-      <c r="B54" s="75"/>
+      <c r="A54" s="74"/>
+      <c r="B54" s="78"/>
       <c r="C54" t="s">
         <v>82</v>
       </c>
@@ -2681,8 +2681,8 @@
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="72"/>
-      <c r="B55" s="78"/>
+      <c r="A55" s="75"/>
+      <c r="B55" s="81"/>
       <c r="C55" s="14" t="s">
         <v>17</v>
       </c>
@@ -2697,7 +2697,7 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="70" t="s">
+      <c r="A56" s="73" t="s">
         <v>90</v>
       </c>
       <c r="B56" s="16" t="s">
@@ -2717,7 +2717,7 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="71"/>
+      <c r="A57" s="74"/>
       <c r="B57" s="17" t="s">
         <v>93</v>
       </c>
@@ -2735,7 +2735,7 @@
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="72"/>
+      <c r="A58" s="75"/>
       <c r="B58" s="1" t="s">
         <v>94</v>
       </c>
@@ -2810,7 +2810,7 @@
       <c r="A2" s="92" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="96" t="s">
+      <c r="B2" s="95" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="28" t="s">
@@ -2826,7 +2826,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="94"/>
-      <c r="B3" s="98"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="12" t="s">
         <v>136</v>
       </c>
@@ -2840,7 +2840,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="94"/>
-      <c r="B4" s="98"/>
+      <c r="B4" s="89"/>
       <c r="C4" s="12" t="s">
         <v>102</v>
       </c>
@@ -2854,7 +2854,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="94"/>
-      <c r="B5" s="98"/>
+      <c r="B5" s="89"/>
       <c r="C5" s="12" t="s">
         <v>172</v>
       </c>
@@ -2868,7 +2868,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="94"/>
-      <c r="B6" s="98"/>
+      <c r="B6" s="89"/>
       <c r="C6" s="12" t="s">
         <v>184</v>
       </c>
@@ -2882,7 +2882,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="94"/>
-      <c r="B7" s="98"/>
+      <c r="B7" s="89"/>
       <c r="C7" s="12" t="s">
         <v>202</v>
       </c>
@@ -2896,7 +2896,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="94"/>
-      <c r="B8" s="98"/>
+      <c r="B8" s="89"/>
       <c r="C8" s="12" t="s">
         <v>251</v>
       </c>
@@ -2910,7 +2910,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="94"/>
-      <c r="B9" s="98"/>
+      <c r="B9" s="89"/>
       <c r="C9" s="12" t="s">
         <v>216</v>
       </c>
@@ -2924,7 +2924,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="94"/>
-      <c r="B10" s="98"/>
+      <c r="B10" s="89"/>
       <c r="C10" s="12" t="s">
         <v>241</v>
       </c>
@@ -2938,12 +2938,12 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="94"/>
-      <c r="B11" s="98"/>
+      <c r="B11" s="89"/>
       <c r="E11" s="35"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="94"/>
-      <c r="B12" s="100" t="s">
+      <c r="B12" s="88" t="s">
         <v>3</v>
       </c>
       <c r="C12" s="37" t="s">
@@ -2959,7 +2959,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="94"/>
-      <c r="B13" s="98"/>
+      <c r="B13" s="89"/>
       <c r="C13" s="12" t="s">
         <v>177</v>
       </c>
@@ -2973,7 +2973,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="94"/>
-      <c r="B14" s="98"/>
+      <c r="B14" s="89"/>
       <c r="C14" s="12" t="s">
         <v>180</v>
       </c>
@@ -2987,7 +2987,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="94"/>
-      <c r="B15" s="98"/>
+      <c r="B15" s="89"/>
       <c r="C15" s="12" t="s">
         <v>181</v>
       </c>
@@ -3001,7 +3001,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="94"/>
-      <c r="B16" s="98"/>
+      <c r="B16" s="89"/>
       <c r="C16" s="12" t="s">
         <v>102</v>
       </c>
@@ -3015,7 +3015,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="94"/>
-      <c r="B17" s="98"/>
+      <c r="B17" s="89"/>
       <c r="C17" s="12" t="s">
         <v>184</v>
       </c>
@@ -3029,7 +3029,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="94"/>
-      <c r="B18" s="98"/>
+      <c r="B18" s="89"/>
       <c r="C18" s="12" t="s">
         <v>202</v>
       </c>
@@ -3043,7 +3043,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="94"/>
-      <c r="B19" s="98"/>
+      <c r="B19" s="89"/>
       <c r="C19" s="12" t="s">
         <v>251</v>
       </c>
@@ -3057,7 +3057,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="94"/>
-      <c r="B20" s="98"/>
+      <c r="B20" s="89"/>
       <c r="C20" s="12" t="s">
         <v>216</v>
       </c>
@@ -3071,7 +3071,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="94"/>
-      <c r="B21" s="98"/>
+      <c r="B21" s="89"/>
       <c r="C21" s="12" t="s">
         <v>241</v>
       </c>
@@ -3085,7 +3085,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="94"/>
-      <c r="B22" s="99"/>
+      <c r="B22" s="91"/>
       <c r="C22" s="39"/>
       <c r="D22" s="39"/>
       <c r="E22" s="40"/>
@@ -3093,7 +3093,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="94"/>
-      <c r="B23" s="89" t="s">
+      <c r="B23" s="96" t="s">
         <v>4</v>
       </c>
       <c r="C23" s="12" t="s">
@@ -3109,7 +3109,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="94"/>
-      <c r="B24" s="89"/>
+      <c r="B24" s="96"/>
       <c r="C24" s="12" t="s">
         <v>136</v>
       </c>
@@ -3123,7 +3123,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="94"/>
-      <c r="B25" s="89"/>
+      <c r="B25" s="96"/>
       <c r="C25" s="12" t="s">
         <v>102</v>
       </c>
@@ -3137,7 +3137,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="94"/>
-      <c r="B26" s="89"/>
+      <c r="B26" s="96"/>
       <c r="C26" s="12" t="s">
         <v>174</v>
       </c>
@@ -3151,7 +3151,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="94"/>
-      <c r="B27" s="89"/>
+      <c r="B27" s="96"/>
       <c r="C27" s="12" t="s">
         <v>184</v>
       </c>
@@ -3165,7 +3165,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="94"/>
-      <c r="B28" s="89"/>
+      <c r="B28" s="96"/>
       <c r="C28" s="12" t="s">
         <v>202</v>
       </c>
@@ -3179,7 +3179,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="94"/>
-      <c r="B29" s="89"/>
+      <c r="B29" s="96"/>
       <c r="C29" s="12" t="s">
         <v>251</v>
       </c>
@@ -3193,7 +3193,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="94"/>
-      <c r="B30" s="89"/>
+      <c r="B30" s="96"/>
       <c r="C30" s="12" t="s">
         <v>216</v>
       </c>
@@ -3207,7 +3207,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="94"/>
-      <c r="B31" s="89"/>
+      <c r="B31" s="96"/>
       <c r="C31" s="12" t="s">
         <v>241</v>
       </c>
@@ -3221,14 +3221,14 @@
     </row>
     <row r="32" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="94"/>
-      <c r="B32" s="89"/>
+      <c r="B32" s="96"/>
       <c r="E32" s="35"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="92" t="s">
         <v>85</v>
       </c>
-      <c r="B33" s="101" t="s">
+      <c r="B33" s="98" t="s">
         <v>5</v>
       </c>
       <c r="C33" s="28" t="s">
@@ -3244,7 +3244,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="94"/>
-      <c r="B34" s="89"/>
+      <c r="B34" s="96"/>
       <c r="C34" s="12" t="s">
         <v>140</v>
       </c>
@@ -3258,7 +3258,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="94"/>
-      <c r="B35" s="89"/>
+      <c r="B35" s="96"/>
       <c r="C35" s="12" t="s">
         <v>169</v>
       </c>
@@ -3272,7 +3272,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="94"/>
-      <c r="B36" s="89"/>
+      <c r="B36" s="96"/>
       <c r="C36" s="12" t="s">
         <v>170</v>
       </c>
@@ -3286,7 +3286,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="94"/>
-      <c r="B37" s="89"/>
+      <c r="B37" s="96"/>
       <c r="C37" s="12" t="s">
         <v>184</v>
       </c>
@@ -3300,7 +3300,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="94"/>
-      <c r="B38" s="89"/>
+      <c r="B38" s="96"/>
       <c r="C38" s="12" t="s">
         <v>202</v>
       </c>
@@ -3314,7 +3314,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="94"/>
-      <c r="B39" s="89"/>
+      <c r="B39" s="96"/>
       <c r="C39" s="12" t="s">
         <v>251</v>
       </c>
@@ -3328,7 +3328,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="94"/>
-      <c r="B40" s="89"/>
+      <c r="B40" s="96"/>
       <c r="C40" s="12" t="s">
         <v>216</v>
       </c>
@@ -3342,7 +3342,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="94"/>
-      <c r="B41" s="89"/>
+      <c r="B41" s="96"/>
       <c r="C41" s="12" t="s">
         <v>241</v>
       </c>
@@ -3356,12 +3356,12 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="94"/>
-      <c r="B42" s="89"/>
+      <c r="B42" s="96"/>
       <c r="E42" s="35"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="94"/>
-      <c r="B43" s="88" t="s">
+      <c r="B43" s="99" t="s">
         <v>8</v>
       </c>
       <c r="C43" s="37" t="s">
@@ -3377,7 +3377,7 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="94"/>
-      <c r="B44" s="89"/>
+      <c r="B44" s="96"/>
       <c r="C44" s="12" t="s">
         <v>142</v>
       </c>
@@ -3391,7 +3391,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="94"/>
-      <c r="B45" s="98"/>
+      <c r="B45" s="89"/>
       <c r="C45" s="12" t="s">
         <v>140</v>
       </c>
@@ -3405,7 +3405,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="94"/>
-      <c r="B46" s="98"/>
+      <c r="B46" s="89"/>
       <c r="C46" s="12" t="s">
         <v>136</v>
       </c>
@@ -3419,7 +3419,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="94"/>
-      <c r="B47" s="98"/>
+      <c r="B47" s="89"/>
       <c r="C47" s="12" t="s">
         <v>157</v>
       </c>
@@ -3433,7 +3433,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="94"/>
-      <c r="B48" s="98"/>
+      <c r="B48" s="89"/>
       <c r="C48" s="12" t="s">
         <v>158</v>
       </c>
@@ -3447,7 +3447,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="94"/>
-      <c r="B49" s="98"/>
+      <c r="B49" s="89"/>
       <c r="C49" s="12" t="s">
         <v>184</v>
       </c>
@@ -3461,7 +3461,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="94"/>
-      <c r="B50" s="98"/>
+      <c r="B50" s="89"/>
       <c r="C50" s="12" t="s">
         <v>202</v>
       </c>
@@ -3475,7 +3475,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="94"/>
-      <c r="B51" s="98"/>
+      <c r="B51" s="89"/>
       <c r="C51" s="12" t="s">
         <v>251</v>
       </c>
@@ -3489,7 +3489,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="94"/>
-      <c r="B52" s="98"/>
+      <c r="B52" s="89"/>
       <c r="C52" s="12" t="s">
         <v>216</v>
       </c>
@@ -3503,7 +3503,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="94"/>
-      <c r="B53" s="98"/>
+      <c r="B53" s="89"/>
       <c r="C53" s="12" t="s">
         <v>241</v>
       </c>
@@ -3516,8 +3516,8 @@
       </c>
     </row>
     <row r="54" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="95"/>
-      <c r="B54" s="102"/>
+      <c r="A54" s="97"/>
+      <c r="B54" s="100"/>
       <c r="C54" s="43"/>
       <c r="D54" s="43"/>
       <c r="E54" s="44"/>
@@ -3527,7 +3527,7 @@
       <c r="A55" s="92" t="s">
         <v>86</v>
       </c>
-      <c r="B55" s="96" t="s">
+      <c r="B55" s="95" t="s">
         <v>87</v>
       </c>
       <c r="C55" s="28" t="s">
@@ -3543,7 +3543,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="94"/>
-      <c r="B56" s="98"/>
+      <c r="B56" s="89"/>
       <c r="C56" s="12" t="s">
         <v>200</v>
       </c>
@@ -3557,12 +3557,12 @@
     </row>
     <row r="57" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="94"/>
-      <c r="B57" s="99"/>
+      <c r="B57" s="91"/>
       <c r="E57" s="33"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="94"/>
-      <c r="B58" s="85" t="s">
+      <c r="B58" s="101" t="s">
         <v>305</v>
       </c>
       <c r="C58" s="63" t="s">
@@ -3578,7 +3578,7 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="94"/>
-      <c r="B59" s="86"/>
+      <c r="B59" s="102"/>
       <c r="C59" s="65" t="s">
         <v>200</v>
       </c>
@@ -3592,7 +3592,7 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="94"/>
-      <c r="B60" s="87"/>
+      <c r="B60" s="103"/>
       <c r="C60" s="65"/>
       <c r="D60" s="65"/>
       <c r="E60" s="66"/>
@@ -3600,7 +3600,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="94"/>
-      <c r="B61" s="88" t="s">
+      <c r="B61" s="99" t="s">
         <v>6</v>
       </c>
       <c r="C61" s="37" t="s">
@@ -3616,7 +3616,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="94"/>
-      <c r="B62" s="89"/>
+      <c r="B62" s="96"/>
       <c r="C62" s="12" t="s">
         <v>136</v>
       </c>
@@ -3630,7 +3630,7 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="94"/>
-      <c r="B63" s="89"/>
+      <c r="B63" s="96"/>
       <c r="C63" s="12" t="s">
         <v>152</v>
       </c>
@@ -3644,7 +3644,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="94"/>
-      <c r="B64" s="89"/>
+      <c r="B64" s="96"/>
       <c r="C64" s="12" t="s">
         <v>184</v>
       </c>
@@ -3658,7 +3658,7 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="94"/>
-      <c r="B65" s="89"/>
+      <c r="B65" s="96"/>
       <c r="C65" s="12" t="s">
         <v>202</v>
       </c>
@@ -3672,7 +3672,7 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="94"/>
-      <c r="B66" s="89"/>
+      <c r="B66" s="96"/>
       <c r="C66" s="12" t="s">
         <v>210</v>
       </c>
@@ -3686,7 +3686,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="94"/>
-      <c r="B67" s="89"/>
+      <c r="B67" s="96"/>
       <c r="C67" s="12" t="s">
         <v>251</v>
       </c>
@@ -3700,7 +3700,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="94"/>
-      <c r="B68" s="89"/>
+      <c r="B68" s="96"/>
       <c r="C68" s="12" t="s">
         <v>216</v>
       </c>
@@ -3714,7 +3714,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="94"/>
-      <c r="B69" s="89"/>
+      <c r="B69" s="96"/>
       <c r="C69" s="12" t="s">
         <v>241</v>
       </c>
@@ -3728,11 +3728,11 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="94"/>
-      <c r="B70" s="90"/>
+      <c r="B70" s="104"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="94"/>
-      <c r="B71" s="88" t="s">
+      <c r="B71" s="99" t="s">
         <v>7</v>
       </c>
       <c r="C71" s="37" t="s">
@@ -3748,7 +3748,7 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="94"/>
-      <c r="B72" s="89"/>
+      <c r="B72" s="96"/>
       <c r="C72" s="12" t="s">
         <v>137</v>
       </c>
@@ -3762,7 +3762,7 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="94"/>
-      <c r="B73" s="89"/>
+      <c r="B73" s="96"/>
       <c r="C73" s="12" t="s">
         <v>150</v>
       </c>
@@ -3776,7 +3776,7 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="94"/>
-      <c r="B74" s="89"/>
+      <c r="B74" s="96"/>
       <c r="C74" s="12" t="s">
         <v>184</v>
       </c>
@@ -3790,7 +3790,7 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="94"/>
-      <c r="B75" s="89"/>
+      <c r="B75" s="96"/>
       <c r="C75" s="12" t="s">
         <v>202</v>
       </c>
@@ -3804,7 +3804,7 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="94"/>
-      <c r="B76" s="89"/>
+      <c r="B76" s="96"/>
       <c r="C76" s="12" t="s">
         <v>210</v>
       </c>
@@ -3818,7 +3818,7 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="94"/>
-      <c r="B77" s="89"/>
+      <c r="B77" s="96"/>
       <c r="C77" s="12" t="s">
         <v>251</v>
       </c>
@@ -3832,7 +3832,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="94"/>
-      <c r="B78" s="89"/>
+      <c r="B78" s="96"/>
       <c r="C78" s="12" t="s">
         <v>216</v>
       </c>
@@ -3846,7 +3846,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="94"/>
-      <c r="B79" s="89"/>
+      <c r="B79" s="96"/>
       <c r="C79" s="12" t="s">
         <v>241</v>
       </c>
@@ -3859,14 +3859,14 @@
       </c>
     </row>
     <row r="80" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A80" s="95"/>
-      <c r="B80" s="91"/>
+      <c r="A80" s="97"/>
+      <c r="B80" s="105"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="92" t="s">
         <v>90</v>
       </c>
-      <c r="B81" s="96" t="s">
+      <c r="B81" s="95" t="s">
         <v>87</v>
       </c>
       <c r="C81" s="28" t="s">
@@ -3882,7 +3882,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="93"/>
-      <c r="B82" s="97"/>
+      <c r="B82" s="90"/>
       <c r="C82" s="55" t="s">
         <v>293</v>
       </c>
@@ -3896,7 +3896,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="94"/>
-      <c r="B83" s="98"/>
+      <c r="B83" s="89"/>
       <c r="C83" s="12" t="s">
         <v>196</v>
       </c>
@@ -3910,12 +3910,12 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="94"/>
-      <c r="B84" s="99"/>
+      <c r="B84" s="91"/>
       <c r="E84" s="35"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="94"/>
-      <c r="B85" s="100" t="s">
+      <c r="B85" s="88" t="s">
         <v>93</v>
       </c>
       <c r="C85" s="37" t="s">
@@ -3931,7 +3931,7 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="94"/>
-      <c r="B86" s="98"/>
+      <c r="B86" s="89"/>
       <c r="C86" s="12" t="s">
         <v>197</v>
       </c>
@@ -3945,7 +3945,7 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="94"/>
-      <c r="B87" s="99"/>
+      <c r="B87" s="91"/>
       <c r="C87" s="39"/>
       <c r="D87" s="39"/>
       <c r="E87" s="40"/>
@@ -3953,7 +3953,7 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="94"/>
-      <c r="B88" s="100" t="s">
+      <c r="B88" s="88" t="s">
         <v>94</v>
       </c>
       <c r="C88" s="12" t="s">
@@ -3969,7 +3969,7 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="94"/>
-      <c r="B89" s="98"/>
+      <c r="B89" s="89"/>
       <c r="C89" s="12" t="s">
         <v>198</v>
       </c>
@@ -3982,8 +3982,8 @@
       </c>
     </row>
     <row r="90" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A90" s="95"/>
-      <c r="B90" s="102"/>
+      <c r="A90" s="97"/>
+      <c r="B90" s="100"/>
       <c r="C90" s="43"/>
       <c r="D90" s="43"/>
       <c r="E90" s="44"/>
@@ -3993,7 +3993,7 @@
       <c r="A91" s="92" t="s">
         <v>212</v>
       </c>
-      <c r="B91" s="96" t="s">
+      <c r="B91" s="95" t="s">
         <v>15</v>
       </c>
       <c r="C91" s="28" t="s">
@@ -4009,7 +4009,7 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="93"/>
-      <c r="B92" s="98"/>
+      <c r="B92" s="89"/>
       <c r="C92" s="12" t="s">
         <v>225</v>
       </c>
@@ -4022,7 +4022,7 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="93"/>
-      <c r="B93" s="99"/>
+      <c r="B93" s="91"/>
       <c r="C93" s="39"/>
       <c r="D93" s="39"/>
       <c r="E93" s="39"/>
@@ -4030,7 +4030,7 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="93"/>
-      <c r="B94" s="100" t="s">
+      <c r="B94" s="88" t="s">
         <v>235</v>
       </c>
       <c r="C94" s="12" t="s">
@@ -4045,7 +4045,7 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="93"/>
-      <c r="B95" s="98"/>
+      <c r="B95" s="89"/>
       <c r="C95" s="12" t="s">
         <v>233</v>
       </c>
@@ -4058,7 +4058,7 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="93"/>
-      <c r="B96" s="98"/>
+      <c r="B96" s="89"/>
       <c r="C96" s="12" t="s">
         <v>229</v>
       </c>
@@ -4071,7 +4071,7 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="93"/>
-      <c r="B97" s="98"/>
+      <c r="B97" s="89"/>
       <c r="C97" s="12" t="s">
         <v>231</v>
       </c>
@@ -4084,7 +4084,7 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="93"/>
-      <c r="B98" s="98"/>
+      <c r="B98" s="89"/>
       <c r="C98" s="12" t="s">
         <v>234</v>
       </c>
@@ -4097,7 +4097,7 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="93"/>
-      <c r="B99" s="98"/>
+      <c r="B99" s="89"/>
       <c r="C99" s="12" t="s">
         <v>244</v>
       </c>
@@ -4110,7 +4110,7 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="93"/>
-      <c r="B100" s="100" t="s">
+      <c r="B100" s="88" t="s">
         <v>265</v>
       </c>
       <c r="C100" s="37" t="s">
@@ -4126,7 +4126,7 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="93"/>
-      <c r="B101" s="97"/>
+      <c r="B101" s="90"/>
       <c r="C101" s="55" t="s">
         <v>261</v>
       </c>
@@ -4140,7 +4140,7 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="93"/>
-      <c r="B102" s="97"/>
+      <c r="B102" s="90"/>
       <c r="C102" s="55" t="s">
         <v>276</v>
       </c>
@@ -4154,7 +4154,7 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="93"/>
-      <c r="B103" s="97"/>
+      <c r="B103" s="90"/>
       <c r="C103" s="55" t="s">
         <v>262</v>
       </c>
@@ -4168,7 +4168,7 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="93"/>
-      <c r="B104" s="97"/>
+      <c r="B104" s="90"/>
       <c r="C104" s="55" t="s">
         <v>278</v>
       </c>
@@ -4182,7 +4182,7 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="93"/>
-      <c r="B105" s="97"/>
+      <c r="B105" s="90"/>
       <c r="C105" s="55" t="s">
         <v>282</v>
       </c>
@@ -4196,7 +4196,7 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" s="93"/>
-      <c r="B106" s="97"/>
+      <c r="B106" s="90"/>
       <c r="C106" s="55" t="s">
         <v>259</v>
       </c>
@@ -4210,7 +4210,7 @@
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" s="93"/>
-      <c r="B107" s="97"/>
+      <c r="B107" s="90"/>
       <c r="C107" s="55" t="s">
         <v>263</v>
       </c>
@@ -4224,7 +4224,7 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="93"/>
-      <c r="B108" s="97"/>
+      <c r="B108" s="90"/>
       <c r="C108" s="55" t="s">
         <v>264</v>
       </c>
@@ -4238,7 +4238,7 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="93"/>
-      <c r="B109" s="100" t="s">
+      <c r="B109" s="88" t="s">
         <v>283</v>
       </c>
       <c r="C109" s="37" t="s">
@@ -4254,7 +4254,7 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="93"/>
-      <c r="B110" s="97"/>
+      <c r="B110" s="90"/>
       <c r="C110" s="55" t="s">
         <v>286</v>
       </c>
@@ -4268,7 +4268,7 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="93"/>
-      <c r="B111" s="97"/>
+      <c r="B111" s="90"/>
       <c r="C111" s="55" t="s">
         <v>288</v>
       </c>
@@ -4282,7 +4282,7 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="93"/>
-      <c r="B112" s="97"/>
+      <c r="B112" s="90"/>
       <c r="C112" s="12" t="s">
         <v>289</v>
       </c>
@@ -4295,11 +4295,11 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="93"/>
-      <c r="B113" s="99"/>
+      <c r="B113" s="91"/>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="93"/>
-      <c r="B114" s="100" t="s">
+      <c r="B114" s="88" t="s">
         <v>294</v>
       </c>
       <c r="C114" s="37" t="s">
@@ -4315,7 +4315,7 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="93"/>
-      <c r="B115" s="98"/>
+      <c r="B115" s="89"/>
       <c r="C115" s="12" t="s">
         <v>297</v>
       </c>
@@ -4331,6 +4331,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="B61:B70"/>
+    <mergeCell ref="B71:B80"/>
+    <mergeCell ref="A81:A90"/>
+    <mergeCell ref="B81:B84"/>
+    <mergeCell ref="B85:B87"/>
     <mergeCell ref="B114:B115"/>
     <mergeCell ref="B109:B113"/>
     <mergeCell ref="A91:A116"/>
@@ -4347,12 +4353,6 @@
     <mergeCell ref="B100:B108"/>
     <mergeCell ref="B91:B93"/>
     <mergeCell ref="A55:A80"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="B61:B70"/>
-    <mergeCell ref="B71:B80"/>
-    <mergeCell ref="A81:A90"/>
-    <mergeCell ref="B81:B84"/>
-    <mergeCell ref="B85:B87"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>